<commit_message>
282-291 mavzulari, barcha 291 ta jadval tayyor (jami 2974 savol) + yakuniy hisobot
</commit_message>
<xml_diff>
--- a/Тест2/205.xlsx
+++ b/Тест2/205.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="76">
   <si>
     <t xml:space="preserve">Question</t>
   </si>
@@ -84,7 +84,13 @@
     <t xml:space="preserve">Endemik qaytalama tifning vektori qaysi?</t>
   </si>
   <si>
-    <t xml:space="preserve">Odam biti (Pediculus)</t>
+    <t xml:space="preserve">Burga (Xenopsylla cheopis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chivin (Anopheles maculipennis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pashsha (Musca domestica)</t>
   </si>
   <si>
     <t xml:space="preserve">To'g'ri javob: Yumshoq kana (Ornithodoros). Endemik shakl uchun asosiy vektorlar Ornithodoros avlodiga mansub yumshoq kanalar. Manba: Mavzu materiali (205.docx); Riedel S. va boshq. Jawetz, Melnick &amp; Adelberg's Medical Microbiology, 28-nashr (2019); WHO. Guidelines for drinking-water quality, 4-nashr, 1-ilova bilan (2017).</t>
@@ -240,16 +246,16 @@
     <t xml:space="preserve">Endemik shakl odamga qaysi sharoitda yuqadi?</t>
   </si>
   <si>
-    <t xml:space="preserve">Maktabda dars paytida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bozorda xarid qilganda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hammom ichida cho'milganda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teatrda o'tirganda</t>
+    <t xml:space="preserve">Maktabda dars o'tirganda, yozganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bozorda xarid qilganda, savdolashganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hammomda cho'milganda, suv ichganda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teatrda tomosha qilganda, o'tirganda</t>
   </si>
   <si>
     <t xml:space="preserve">O'choqqa kirganda, kana chaqqanda</t>
@@ -706,230 +712,230 @@
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>